<commit_message>
samples: demonstrate date text formatting
</commit_message>
<xml_diff>
--- a/samples/scalar_values_output.xlsx
+++ b/samples/scalar_values_output.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -647,81 +647,115 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Boolean</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="b">
-        <v>1</v>
+          <t>Date text filter</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>native boolean</t>
+          <t>explicit text: 2026-08</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Mixed text</t>
+          <t>Date in sentence</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Invoice INV-1042</t>
+          <t>For the month ending 19 August 2026</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>always text</t>
+          <t>formatted text in mixed content</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Upper filter</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>ACME INDUSTRIES</t>
-        </is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>uppercase text</t>
+          <t>native boolean</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Join filter</t>
+          <t>Mixed text</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>priority / renewal</t>
+          <t>Invoice INV-1042</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>one text value</t>
+          <t>always text</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
+          <t>Upper filter</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>ACME INDUSTRIES</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>uppercase text</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Join filter</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>priority / renewal</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>one text value</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
           <t>Default filter</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>not supplied</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>explicit fallback</t>
         </is>

</xml_diff>

<commit_message>
samples: demonstrate numeric sum filters
</commit_message>
<xml_diff>
--- a/samples/scalar_values_output.xlsx
+++ b/samples/scalar_values_output.xlsx
@@ -144,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -167,6 +167,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -534,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -747,15 +750,45 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
+          <t>Numeric sum</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>nulls skipped; native number: 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Record-column sum</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>literal column key; native number: 150</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
           <t>Default filter</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>not supplied</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>explicit fallback</t>
         </is>

</xml_diff>

<commit_message>
docs: demonstrate aggregate and arithmetic expressions
</commit_message>
<xml_diff>
--- a/samples/scalar_values_output.xlsx
+++ b/samples/scalar_values_output.xlsx
@@ -537,12 +537,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -557,7 +557,7 @@
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Single-expression cells preserve types; mixed content becomes text; filters are explicit.</t>
+          <t>Typed expressions support explicit filters, collection aggregates, and basic arithmetic.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -780,15 +780,105 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
+          <t>Record-column minimum</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>nulls skipped: 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Record-column maximum</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>nulls skipped: 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Record count</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>all records counted: 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Aggregate arithmetic</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>parenthesized filtered operands: 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Basic arithmetic</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>standard precedence: 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Unary signs</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>native number: 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
           <t>Default filter</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>not supplied</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>explicit fallback</t>
         </is>

</xml_diff>